<commit_message>
Update Lab 0 documentation, verification, and gitignore
</commit_message>
<xml_diff>
--- a/module1/lab0_basics/documentation/lab0_deployment_tracking.xlsx
+++ b/module1/lab0_basics/documentation/lab0_deployment_tracking.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/7d013bf0b423e019/Desktop/1536 Stuff/!!Cloud Engineer/Theo Class/Class 8/SEIR 10.13.2026/HW_Class8-Week1/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cdela\Documents\TheoWAF\class8\SEIR_Foundations\seir-foundations-labs\module1\lab0_basics\documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="156" documentId="8_{95283C39-ACB0-4DCB-937A-855A49A0E1BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AC8511CF-FBB5-4C3E-A3B3-EF8F38E39162}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87DA20BD-BF58-400B-8D32-5CABC477D434}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-150" windowWidth="29040" windowHeight="15720" xr2:uid="{30705D01-5DBF-4AC3-BFE1-436EDED0B5AA}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{30705D01-5DBF-4AC3-BFE1-436EDED0B5AA}"/>
   </bookViews>
   <sheets>
     <sheet name="Evidence Table" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,6 @@
     <sheet name="Deployment 4" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -265,6 +264,18 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -276,18 +287,6 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -813,10 +812,6 @@
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1149,102 +1144,102 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" s="2" customFormat="1" ht="30" x14ac:dyDescent="0.25">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="8" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="8" t="s">
+      <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="8" t="s">
+      <c r="D1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="8" t="s">
+      <c r="E1" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="8" t="s">
+      <c r="F1" s="4" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="153.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="9">
+      <c r="A2" s="5">
         <v>1</v>
       </c>
-      <c r="B2" s="9" t="s">
+      <c r="B2" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="9" t="s">
+      <c r="C2" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="10" t="s">
+      <c r="D2" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="E2" s="9" t="s">
+      <c r="E2" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="F2" s="11" t="s">
+      <c r="F2" s="7" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="75" x14ac:dyDescent="0.25">
-      <c r="A3" s="9">
+      <c r="A3" s="5">
         <v>2</v>
       </c>
-      <c r="B3" s="9" t="s">
+      <c r="B3" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="9" t="s">
+      <c r="C3" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="D3" s="10" t="s">
+      <c r="D3" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="E3" s="9" t="s">
+      <c r="E3" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="F3" s="9" t="s">
+      <c r="F3" s="5" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="90" x14ac:dyDescent="0.25">
-      <c r="A4" s="9">
+      <c r="A4" s="5">
         <v>3</v>
       </c>
-      <c r="B4" s="9" t="s">
+      <c r="B4" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="C4" s="9" t="s">
+      <c r="C4" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="D4" s="10" t="s">
+      <c r="D4" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="E4" s="9" t="s">
+      <c r="E4" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="F4" s="9" t="s">
+      <c r="F4" s="5" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="90" x14ac:dyDescent="0.25">
-      <c r="A5" s="9">
+      <c r="A5" s="5">
         <v>4</v>
       </c>
-      <c r="B5" s="9" t="s">
+      <c r="B5" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="C5" s="9" t="s">
+      <c r="C5" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="D5" s="10" t="s">
+      <c r="D5" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="E5" s="9" t="s">
+      <c r="E5" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="F5" s="9" t="s">
+      <c r="F5" s="5" t="s">
         <v>18</v>
       </c>
     </row>
@@ -1256,6 +1251,7 @@
     <hyperlink ref="D5" location="'Deployment 4'!A1" display="Deployment 4" xr:uid="{289CB7A1-3F73-4BF8-8FF5-872610E37991}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup scale="54" orientation="landscape" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1265,26 +1261,26 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="2" spans="4:20" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="D2" s="4" t="s">
+      <c r="D2" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="E2" s="4"/>
-      <c r="F2" s="4"/>
-      <c r="G2" s="4"/>
-      <c r="H2" s="4"/>
-      <c r="I2" s="4"/>
-      <c r="J2" s="4"/>
-      <c r="K2" s="4"/>
-      <c r="L2" s="4"/>
-      <c r="M2" s="4"/>
-      <c r="N2" s="4"/>
-      <c r="O2" s="4"/>
-      <c r="Q2" s="5" t="s">
+      <c r="E2" s="8"/>
+      <c r="F2" s="8"/>
+      <c r="G2" s="8"/>
+      <c r="H2" s="8"/>
+      <c r="I2" s="8"/>
+      <c r="J2" s="8"/>
+      <c r="K2" s="8"/>
+      <c r="L2" s="8"/>
+      <c r="M2" s="8"/>
+      <c r="N2" s="8"/>
+      <c r="O2" s="8"/>
+      <c r="Q2" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="R2" s="6"/>
-      <c r="S2" s="6"/>
-      <c r="T2" s="7"/>
+      <c r="R2" s="10"/>
+      <c r="S2" s="10"/>
+      <c r="T2" s="11"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1295,7 +1291,11 @@
     <hyperlink ref="Q2:T2" location="'Evidence Table'!A1" display="Return to  Evidence Table" xr:uid="{C189A6C2-8841-45B8-9799-19A086EDB749}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
+  <pageSetup scale="44" orientation="portrait" r:id="rId1"/>
+  <rowBreaks count="1" manualBreakCount="1">
+    <brk id="48" max="16383" man="1"/>
+  </rowBreaks>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -1305,26 +1305,26 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="2" spans="4:21" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="D2" s="4" t="s">
+      <c r="D2" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="E2" s="4"/>
-      <c r="F2" s="4"/>
-      <c r="G2" s="4"/>
-      <c r="H2" s="4"/>
-      <c r="I2" s="4"/>
-      <c r="J2" s="4"/>
-      <c r="K2" s="4"/>
-      <c r="L2" s="4"/>
-      <c r="M2" s="4"/>
-      <c r="N2" s="4"/>
-      <c r="O2" s="4"/>
-      <c r="R2" s="5" t="s">
+      <c r="E2" s="8"/>
+      <c r="F2" s="8"/>
+      <c r="G2" s="8"/>
+      <c r="H2" s="8"/>
+      <c r="I2" s="8"/>
+      <c r="J2" s="8"/>
+      <c r="K2" s="8"/>
+      <c r="L2" s="8"/>
+      <c r="M2" s="8"/>
+      <c r="N2" s="8"/>
+      <c r="O2" s="8"/>
+      <c r="R2" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="S2" s="6"/>
-      <c r="T2" s="6"/>
-      <c r="U2" s="7"/>
+      <c r="S2" s="10"/>
+      <c r="T2" s="10"/>
+      <c r="U2" s="11"/>
     </row>
     <row r="3" spans="4:21" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="D3" s="3"/>
@@ -1349,7 +1349,8 @@
     <hyperlink ref="R2:U2" location="'Evidence Table'!A1" display="Return to  Evidence Table" xr:uid="{EC90D2B9-D474-4EBC-A01F-DFAD19671A62}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
+  <pageSetup scale="34" orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -1359,26 +1360,26 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="2" spans="4:21" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="D2" s="4" t="s">
+      <c r="D2" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="E2" s="4"/>
-      <c r="F2" s="4"/>
-      <c r="G2" s="4"/>
-      <c r="H2" s="4"/>
-      <c r="I2" s="4"/>
-      <c r="J2" s="4"/>
-      <c r="K2" s="4"/>
-      <c r="L2" s="4"/>
-      <c r="M2" s="4"/>
-      <c r="N2" s="4"/>
-      <c r="O2" s="4"/>
-      <c r="R2" s="5" t="s">
+      <c r="E2" s="8"/>
+      <c r="F2" s="8"/>
+      <c r="G2" s="8"/>
+      <c r="H2" s="8"/>
+      <c r="I2" s="8"/>
+      <c r="J2" s="8"/>
+      <c r="K2" s="8"/>
+      <c r="L2" s="8"/>
+      <c r="M2" s="8"/>
+      <c r="N2" s="8"/>
+      <c r="O2" s="8"/>
+      <c r="R2" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="S2" s="6"/>
-      <c r="T2" s="6"/>
-      <c r="U2" s="7"/>
+      <c r="S2" s="10"/>
+      <c r="T2" s="10"/>
+      <c r="U2" s="11"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1389,7 +1390,8 @@
     <hyperlink ref="R2:U2" location="'Evidence Table'!A1" display="Return to  Evidence Table" xr:uid="{885D37DA-B77B-4B20-8978-1D4FEB2FB9A4}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
+  <pageSetup scale="36" orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -1399,26 +1401,26 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="2" spans="4:19" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="D2" s="4" t="s">
+      <c r="D2" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="E2" s="4"/>
-      <c r="F2" s="4"/>
-      <c r="G2" s="4"/>
-      <c r="H2" s="4"/>
-      <c r="I2" s="4"/>
-      <c r="J2" s="4"/>
-      <c r="K2" s="4"/>
-      <c r="L2" s="4"/>
-      <c r="M2" s="4"/>
-      <c r="N2" s="4"/>
-      <c r="O2" s="4"/>
-      <c r="P2" s="5" t="s">
+      <c r="E2" s="8"/>
+      <c r="F2" s="8"/>
+      <c r="G2" s="8"/>
+      <c r="H2" s="8"/>
+      <c r="I2" s="8"/>
+      <c r="J2" s="8"/>
+      <c r="K2" s="8"/>
+      <c r="L2" s="8"/>
+      <c r="M2" s="8"/>
+      <c r="N2" s="8"/>
+      <c r="O2" s="8"/>
+      <c r="P2" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="Q2" s="6"/>
-      <c r="R2" s="6"/>
-      <c r="S2" s="7"/>
+      <c r="Q2" s="10"/>
+      <c r="R2" s="10"/>
+      <c r="S2" s="11"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1429,6 +1431,7 @@
     <hyperlink ref="P2:S2" location="'Evidence Table'!A1" display="Return to  Evidence Table" xr:uid="{0A8D9239-CA85-4A3D-A1CC-76960C9D6874}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
+  <pageSetup scale="51" orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>